<commit_message>
Add Value to items
</commit_message>
<xml_diff>
--- a/rogue-boi-core/assets/game-config.xlsx
+++ b/rogue-boi-core/assets/game-config.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="114">
   <si>
     <t xml:space="preserve">tag</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t xml:space="preserve">aoe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
   </si>
   <si>
     <t xml:space="preserve">Stairs</t>
@@ -456,12 +459,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -646,51 +649,53 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3"/>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>10</v>
@@ -707,44 +712,44 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>100</v>
@@ -764,19 +769,19 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>35</v>
@@ -796,59 +801,65 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J9" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="P9" s="0" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="J10" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="P10" s="0" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>4</v>
@@ -856,22 +867,25 @@
       <c r="I11" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="P11" s="0" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H12" s="1" t="n">
         <v>2</v>
@@ -879,43 +893,49 @@
       <c r="I12" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="P12" s="0" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D13" s="1" t="str">
         <f aca="false">"Restores "&amp;K13&amp;" health"</f>
         <v>Restores 3 health</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K13" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="P13" s="0" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L14" s="1" t="n">
         <v>3</v>
@@ -926,22 +946,25 @@
       <c r="N14" s="1" t="n">
         <v>4</v>
       </c>
+      <c r="P14" s="0" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L15" s="1" t="n">
         <v>10</v>
@@ -952,23 +975,26 @@
       <c r="N15" s="1" t="n">
         <v>4</v>
       </c>
+      <c r="P15" s="0" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D16" s="1" t="str">
         <f aca="false">"Hurl a fireball dealing damage in an area with radius "&amp;O16&amp;" for "&amp;L16&amp;" damage"</f>
         <v>Hurl a fireball dealing damage in an area with radius 3 for 4 damage</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L16" s="1" t="n">
         <v>4</v>
@@ -982,22 +1008,25 @@
       <c r="O16" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="P16" s="0" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>200</v>
@@ -1017,19 +1046,19 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>75</v>
-      </c>
       <c r="D18" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>25</v>
@@ -1049,19 +1078,19 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>80</v>
+      <c r="D19" s="3" t="s">
+        <v>81</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F19" s="1" t="n">
         <f aca="false">_xlfn.CEILING.MATH(F7*2/3)+5</f>
@@ -1085,19 +1114,19 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>84</v>
+      <c r="D20" s="3" t="s">
+        <v>85</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>120</v>
@@ -1117,19 +1146,19 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>1</v>
@@ -1137,25 +1166,28 @@
       <c r="M21" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="N21" s="3" t="n">
+      <c r="N21" s="4" t="n">
         <v>4</v>
+      </c>
+      <c r="P21" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H22" s="1" t="n">
         <v>7</v>
@@ -1163,22 +1195,25 @@
       <c r="I22" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="P22" s="0" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H23" s="1" t="n">
         <f aca="false">_xlfn.FLOOR.MATH((H22+H11)/2)</f>
@@ -1187,22 +1222,25 @@
       <c r="I23" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="P23" s="0" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="D24" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>50</v>
@@ -1222,60 +1260,63 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J25" s="1"/>
       <c r="L25" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="M25" s="3" t="n">
+      <c r="M25" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="3" t="n">
+      <c r="N25" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="P25" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="D26" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="F26" s="4" t="n">
         <v>500</v>
       </c>
-      <c r="G26" s="0" t="n">
+      <c r="G26" s="4" t="n">
         <v>5000</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="I26" s="0" t="n">
+      <c r="I26" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J26" s="0" t="n">
+      <c r="J26" s="4" t="n">
         <v>1000</v>
       </c>
     </row>
@@ -1300,13 +1341,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1314,7 +1355,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>80</v>
@@ -1325,7 +1366,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>120</v>
@@ -1336,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>15</v>
@@ -1347,7 +1388,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>30</v>
@@ -1358,7 +1399,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>30</v>
@@ -1369,20 +1410,20 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C8" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1391,31 +1432,31 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C10" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C11" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1450,13 +1491,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1464,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>80</v>
@@ -1475,7 +1516,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>40</v>
@@ -1486,7 +1527,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>40</v>
@@ -1497,7 +1538,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>10</v>
@@ -1508,7 +1549,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>30</v>
@@ -1519,7 +1560,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>30</v>
@@ -1530,7 +1571,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>25</v>
@@ -1541,7 +1582,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>25</v>
@@ -1552,7 +1593,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>10</v>
@@ -1563,9 +1604,9 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1574,9 +1615,9 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1585,9 +1626,9 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C13" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1596,9 +1637,9 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C14" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1629,31 +1670,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B2" s="3" t="n">
+      <c r="A2" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B3" s="3" t="n">
+      <c r="A3" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="4" t="n">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add SlowScrolls. Slowed status has a chance to delay movement
</commit_message>
<xml_diff>
--- a/rogue-boi-core/assets/game-config.xlsx
+++ b/rogue-boi-core/assets/game-config.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="stuff-descriptor" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="119">
   <si>
     <t xml:space="preserve">tag</t>
   </si>
@@ -73,6 +73,9 @@
     <t xml:space="preserve">value</t>
   </si>
   <si>
+    <t xml:space="preserve">slow</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stairs</t>
   </si>
   <si>
@@ -350,6 +353,18 @@
   </si>
   <si>
     <t xml:space="preserve">Buy and sell items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SlowScroll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply slow effect to the target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yellow</t>
   </si>
   <si>
     <t xml:space="preserve">level</t>
@@ -459,12 +474,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -487,37 +502,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -590,8 +605,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultColWidth="11.546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Q27"/>
+  <sheetFormatPr defaultColWidth="11.546875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.34"/>
@@ -652,50 +667,53 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>10</v>
@@ -712,44 +730,44 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>100</v>
@@ -769,19 +787,19 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>35</v>
@@ -801,65 +819,65 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P9" s="0" t="n">
+      <c r="P9" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="J10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P10" s="0" t="n">
+      <c r="P10" s="3" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>4</v>
@@ -867,25 +885,25 @@
       <c r="I11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P11" s="0" t="n">
+      <c r="P11" s="3" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H12" s="1" t="n">
         <v>2</v>
@@ -893,49 +911,49 @@
       <c r="I12" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P12" s="0" t="n">
+      <c r="P12" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D13" s="1" t="str">
         <f aca="false">"Restores "&amp;K13&amp;" health"</f>
         <v>Restores 3 health</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K13" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P13" s="0" t="n">
+      <c r="P13" s="3" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="L14" s="1" t="n">
         <v>3</v>
@@ -946,25 +964,25 @@
       <c r="N14" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="P14" s="0" t="n">
+      <c r="P14" s="3" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="L15" s="1" t="n">
         <v>10</v>
@@ -975,26 +993,26 @@
       <c r="N15" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="P15" s="0" t="n">
+      <c r="P15" s="3" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D16" s="1" t="str">
         <f aca="false">"Hurl a fireball dealing damage in an area with radius "&amp;O16&amp;" for "&amp;L16&amp;" damage"</f>
         <v>Hurl a fireball dealing damage in an area with radius 3 for 4 damage</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L16" s="1" t="n">
         <v>4</v>
@@ -1008,25 +1026,25 @@
       <c r="O16" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="P16" s="0" t="n">
+      <c r="P16" s="3" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>200</v>
@@ -1046,19 +1064,19 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="D18" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>25</v>
@@ -1078,19 +1096,19 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>81</v>
+      <c r="D19" s="4" t="s">
+        <v>82</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F19" s="1" t="n">
         <f aca="false">_xlfn.CEILING.MATH(F7*2/3)+5</f>
@@ -1114,19 +1132,19 @@
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>85</v>
+      <c r="D20" s="4" t="s">
+        <v>86</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>120</v>
@@ -1146,19 +1164,19 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>1</v>
@@ -1166,28 +1184,28 @@
       <c r="M21" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="N21" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P21" s="0" t="n">
+      <c r="N21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="P21" s="3" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H22" s="1" t="n">
         <v>7</v>
@@ -1195,25 +1213,25 @@
       <c r="I22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="P22" s="0" t="n">
+      <c r="P22" s="3" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H23" s="1" t="n">
         <f aca="false">_xlfn.FLOOR.MATH((H22+H11)/2)</f>
@@ -1222,25 +1240,25 @@
       <c r="I23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="P23" s="0" t="n">
+      <c r="P23" s="3" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>98</v>
-      </c>
       <c r="D24" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>50</v>
@@ -1260,64 +1278,84 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J25" s="1"/>
       <c r="L25" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="M25" s="4" t="n">
+      <c r="M25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="4" t="n">
+      <c r="N25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="P25" s="0" t="n">
+      <c r="P25" s="3" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="D26" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F26" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" s="3" t="n">
         <v>500</v>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="G26" s="3" t="n">
         <v>5000</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="I26" s="4" t="n">
+      <c r="I26" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J26" s="4" t="n">
+      <c r="J26" s="3" t="n">
         <v>1000</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q27" s="3" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1337,17 +1375,17 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="11.546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.546875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1355,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>80</v>
@@ -1366,7 +1404,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>120</v>
@@ -1377,7 +1415,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>15</v>
@@ -1388,7 +1426,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>30</v>
@@ -1399,7 +1437,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>30</v>
@@ -1410,20 +1448,20 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="C8" s="3" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1432,31 +1470,31 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="3" t="n">
         <v>2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C10" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="C10" s="3" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="C11" s="3" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1482,8 +1520,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="11.546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultColWidth="11.546875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.43"/>
@@ -1491,13 +1529,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1505,7 +1543,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>80</v>
@@ -1516,7 +1554,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>40</v>
@@ -1527,7 +1565,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>40</v>
@@ -1538,7 +1576,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>10</v>
@@ -1549,7 +1587,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>30</v>
@@ -1560,7 +1598,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>30</v>
@@ -1571,7 +1609,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>25</v>
@@ -1582,7 +1620,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>25</v>
@@ -1593,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>10</v>
@@ -1604,9 +1642,9 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="C11" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1615,9 +1653,9 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="C12" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1626,9 +1664,9 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C13" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="C13" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1637,10 +1675,21 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C14" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="C14" s="3" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1666,35 +1715,35 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="10.08203125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.08203125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B2" s="4" t="n">
+      <c r="A2" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="4" t="n">
+      <c r="A3" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="3" t="n">
         <v>90</v>
       </c>
     </row>

</xml_diff>